<commit_message>
Revise Beebop call priorities and share recommendations with Rocksteady
Move EcoFriendly and Select into the first ten, correct the geography rule to a 120-mile radius, and document ranking rationale and historical state-volume limits. Preserve Claude's main workbook.
</commit_message>
<xml_diff>
--- a/Tissue Supplier Research/Beebop/round2-2026-09-28/Tissue_Supplier_Cross_Reference_2026-09-28.xlsx
+++ b/Tissue Supplier Research/Beebop/round2-2026-09-28/Tissue_Supplier_Cross_Reference_2026-09-28.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="The First 10 Revised" sheetId="1" r:id="R94e14cf760e44278"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fact Review" sheetId="2" r:id="R2ec220c5d1f741fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Previous 30 Crosscheck" sheetId="3" r:id="R6f32501d64cd452e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Additional Leads" sheetId="4" r:id="R1c6b315190eb40a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Other Tissue Providers" sheetId="5" r:id="R79e5130b08c94320"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="The First 10 Revised" sheetId="1" r:id="R8541bbdd4f6d4f5a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fact Review" sheetId="2" r:id="R26aa570faa734d86"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Previous 30 Crosscheck" sheetId="3" r:id="Re9561722f7874452"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Additional Leads" sheetId="4" r:id="Re7743bf846a141bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Other Tissue Providers" sheetId="5" r:id="R2acc1031722c4e1f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -21,7 +21,7 @@
     <x:numFmt numFmtId="200" formatCode="0.0"/>
     <x:numFmt numFmtId="201" formatCode="0"/>
   </x:numFmts>
-  <x:fonts count="5">
+  <x:fonts count="7">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -46,6 +46,15 @@
       <x:b/>
       <x:sz val="10"/>
       <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF415B76"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
@@ -78,7 +87,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="20">
+  <x:cellXfs count="26">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -135,6 +144,22 @@
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -146,7 +171,7 @@
         <x:color rgb="FF9D2626"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE5E5"/>
         </x:patternFill>
       </x:fill>
@@ -157,7 +182,7 @@
         <x:color rgb="FF9D2626"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE5E5"/>
         </x:patternFill>
       </x:fill>
@@ -168,7 +193,7 @@
         <x:color rgb="FF825400"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF1D5"/>
         </x:patternFill>
       </x:fill>
@@ -195,8 +220,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="FactReview" displayName="FactReview" ref="A7:H30" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A7:H30"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="FactReview" displayName="FactReview" ref="A7:H33" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A7:H33"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Topic"/>
@@ -497,7 +522,7 @@
     </x:row>
     <x:row r="2" ht="22" customHeight="1">
       <x:c r="A2" s="4" t="str">
-        <x:v>The First 10: revised qualification priorities</x:v>
+        <x:v>The First 10: revised call priorities</x:v>
       </x:c>
       <x:c r="B2" s="5"/>
       <x:c r="C2" s="5"/>
@@ -521,7 +546,7 @@
     </x:row>
     <x:row r="4" ht="22" customHeight="1">
       <x:c r="A4" s="6" t="str">
-        <x:v>Checked September 28, 2026, including Claude’s concurrent update. Unknown means unconfirmed, not zero.</x:v>
+        <x:v>Revision 2.1, September 28, 2026. Documented fit drives priority; missing information earns no advantage.</x:v>
       </x:c>
       <x:c r="B4" s="2"/>
       <x:c r="C4" s="2"/>
@@ -533,7 +558,7 @@
     </x:row>
     <x:row r="5" ht="22" customHeight="1">
       <x:c r="A5" s="6" t="str">
-        <x:v>Distance origin: Durham City Hall. These are qualification calls, not verified Martin’s-scale replacements.</x:v>
+        <x:v>Eligibility: within 120 radial miles of Durham City Hall. Road mileage measures logistics only.</x:v>
       </x:c>
       <x:c r="B5" s="2"/>
       <x:c r="C5" s="2"/>
@@ -579,7 +604,7 @@
         <x:v>Website / public page</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="45" customHeight="1">
+    <x:row r="8" ht="58" customHeight="1">
       <x:c r="A8" s="17" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -599,7 +624,7 @@
         <x:v>336-628-4949</x:v>
       </x:c>
       <x:c r="F8" s="12" t="str">
-        <x:v>Published 150 lb live minimum overlaps the target; custom processing structure.</x:v>
+        <x:v>Published 150-pound live minimum overlaps the target; custom processing and nearby slaughter site.</x:v>
       </x:c>
       <x:c r="G8" s="12" t="str">
         <x:v>Both unknown</x:v>
@@ -608,7 +633,7 @@
         <x:v>https://www.piedmontcustommeats.com/</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="45" customHeight="1">
+    <x:row r="9" ht="58" customHeight="1">
       <x:c r="A9" s="19" t="n">
         <x:v>2</x:v>
       </x:c>
@@ -628,7 +653,7 @@
         <x:v>919-894-2587</x:v>
       </x:c>
       <x:c r="F9" s="11" t="str">
-        <x:v>Nearby inspected swine plant; Lee’s website and contact identity match.</x:v>
+        <x:v>Nearby inspected swine plant with matching company identity. Practical early qualification prospect.</x:v>
       </x:c>
       <x:c r="G9" s="11" t="str">
         <x:v>Both unknown</x:v>
@@ -637,143 +662,143 @@
         <x:v>https://leesfreshmarketnc.com/</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="45" customHeight="1">
+    <x:row r="10" ht="58" customHeight="1">
       <x:c r="A10" s="17" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="B10" s="12" t="str">
-        <x:v>Flowers Slaughter House</x:v>
+        <x:v>Gale McLamb Meats</x:v>
       </x:c>
       <x:c r="C10" s="16" t="n">
         <x:f>INDEX('Previous 30 Crosscheck'!$D$8:$D$37,MATCH($B10,'Previous 30 Crosscheck'!$A$8:$A$37,0))</x:f>
-        <x:v>63.30834178398154</x:v>
+        <x:v>59.73757009067048</x:v>
       </x:c>
       <x:c r="D10" s="16" t="n">
         <x:f>INDEX('Previous 30 Crosscheck'!$E$8:$E$37,MATCH($B10,'Previous 30 Crosscheck'!$A$8:$A$37,0))</x:f>
-        <x:v>51.63749846644421</x:v>
+        <x:v>48.036921080446234</x:v>
       </x:c>
       <x:c r="E10" s="17" t="str">
         <x:f>INDEX('Previous 30 Crosscheck'!$J$8:$J$37,MATCH($B10,'Previous 30 Crosscheck'!$A$8:$A$37,0))</x:f>
-        <x:v>252-237-2982</x:v>
+        <x:v>910-892-7279</x:v>
       </x:c>
       <x:c r="F10" s="12" t="str">
-        <x:v>Nearby hog slaughter lead; duplicate George Flowers entry counted once.</x:v>
+        <x:v>Nearby state-inspected swine slaughter; practical Benson/Dunn visit grouping. No volume advantage assumed.</x:v>
       </x:c>
       <x:c r="G10" s="12" t="str">
         <x:v>Both unknown</x:v>
       </x:c>
       <x:c r="H10" s="12" t="str">
-        <x:v>https://www.facebook.com/p/Flowers-Slaughterhouse-Page-100063690244587/</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="45" customHeight="1">
+        <x:v>No company website confirmed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="58" customHeight="1">
       <x:c r="A11" s="19" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="B11" s="11" t="str">
-        <x:v>Contentnea Farms</x:v>
+        <x:v>EcoFriendly Foods</x:v>
       </x:c>
       <x:c r="C11" s="18" t="n">
-        <x:f>INDEX('Previous 30 Crosscheck'!$D$8:$D$37,MATCH($B11,'Previous 30 Crosscheck'!$A$8:$A$37,0))</x:f>
-        <x:v>90.29008092738407</x:v>
+        <x:f>INDEX('Additional Leads'!$C$8:$C$30,MATCH($B11,'Additional Leads'!$A$8:$A$30,0))</x:f>
+        <x:v>120.44771037143083</x:v>
       </x:c>
       <x:c r="D11" s="18" t="n">
-        <x:f>INDEX('Previous 30 Crosscheck'!$E$8:$E$37,MATCH($B11,'Previous 30 Crosscheck'!$A$8:$A$37,0))</x:f>
-        <x:v>72.64760579541328</x:v>
+        <x:f>INDEX('Additional Leads'!$D$8:$D$30,MATCH($B11,'Additional Leads'!$A$8:$A$30,0))</x:f>
+        <x:v>92.57037085355904</x:v>
       </x:c>
       <x:c r="E11" s="19" t="str">
-        <x:f>INDEX('Previous 30 Crosscheck'!$J$8:$J$37,MATCH($B11,'Previous 30 Crosscheck'!$A$8:$A$37,0))</x:f>
-        <x:v>252-289-3083</x:v>
+        <x:f>INDEX('Additional Leads'!$I$8:$I$30,MATCH($B11,'Additional Leads'!$A$8:$A$30,0))</x:f>
+        <x:v>540-525-0352</x:v>
       </x:c>
       <x:c r="F11" s="11" t="str">
-        <x:v>Current state listing plus company pork-processing evidence.</x:v>
+        <x:v>Custom harvest supports an early supplier-performed collection discussion. Within radius; pig volume unverified.</x:v>
       </x:c>
       <x:c r="G11" s="11" t="str">
-        <x:v>Both unknown</x:v>
+        <x:v>Both unknown; historical state data weaken volume case</x:v>
       </x:c>
       <x:c r="H11" s="11" t="str">
-        <x:v>https://contentneafarms.com/</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="45" customHeight="1">
+        <x:v>https://www.ecofriendly.com/services</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="58" customHeight="1">
       <x:c r="A12" s="17" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="B12" s="12" t="str">
-        <x:v>Farmington Meat Processing</x:v>
+        <x:v>Flowers Slaughter House</x:v>
       </x:c>
       <x:c r="C12" s="16" t="n">
-        <x:f>INDEX('Additional Leads'!$C$8:$C$30,MATCH($B12,'Additional Leads'!$A$8:$A$30,0))</x:f>
-        <x:v>102.58086524695776</x:v>
+        <x:f>INDEX('Previous 30 Crosscheck'!$D$8:$D$37,MATCH($B12,'Previous 30 Crosscheck'!$A$8:$A$37,0))</x:f>
+        <x:v>63.30834178398154</x:v>
       </x:c>
       <x:c r="D12" s="16" t="n">
-        <x:f>INDEX('Additional Leads'!$D$8:$D$30,MATCH($B12,'Additional Leads'!$A$8:$A$30,0))</x:f>
-        <x:v>91.65576089158736</x:v>
+        <x:f>INDEX('Previous 30 Crosscheck'!$E$8:$E$37,MATCH($B12,'Previous 30 Crosscheck'!$A$8:$A$37,0))</x:f>
+        <x:v>51.63749846644421</x:v>
       </x:c>
       <x:c r="E12" s="17" t="str">
-        <x:f>INDEX('Additional Leads'!$I$8:$I$30,MATCH($B12,'Additional Leads'!$A$8:$A$30,0))</x:f>
-        <x:v>336-998-7092</x:v>
+        <x:f>INDEX('Previous 30 Crosscheck'!$J$8:$J$37,MATCH($B12,'Previous 30 Crosscheck'!$A$8:$A$37,0))</x:f>
+        <x:v>252-237-2982</x:v>
       </x:c>
       <x:c r="F12" s="12" t="str">
-        <x:v>Promoted from Claude’s grouped row; state and social evidence agree on pigs.</x:v>
+        <x:v>Nearby documented hog slaughter. George Flowers is the same plant and is counted once.</x:v>
       </x:c>
       <x:c r="G12" s="12" t="str">
         <x:v>Both unknown</x:v>
       </x:c>
       <x:c r="H12" s="12" t="str">
-        <x:v>https://www.facebook.com/FarmingtonMeat/</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="45" customHeight="1">
+        <x:v>https://www.facebook.com/p/Flowers-Slaughterhouse-Page-100063690244587/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="58" customHeight="1">
       <x:c r="A13" s="19" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="B13" s="11" t="str">
-        <x:v>Easternview Farms</x:v>
+        <x:v>Select Meats</x:v>
       </x:c>
       <x:c r="C13" s="18" t="n">
-        <x:f>INDEX('Additional Leads'!$C$8:$C$30,MATCH($B13,'Additional Leads'!$A$8:$A$30,0))</x:f>
-        <x:v>75.973440109759</x:v>
+        <x:f>INDEX('Previous 30 Crosscheck'!$D$8:$D$37,MATCH($B13,'Previous 30 Crosscheck'!$A$8:$A$37,0))</x:f>
+        <x:v>114.4866479758212</x:v>
       </x:c>
       <x:c r="D13" s="18" t="n">
-        <x:f>INDEX('Additional Leads'!$D$8:$D$30,MATCH($B13,'Additional Leads'!$A$8:$A$30,0))</x:f>
-        <x:v>65.18257538646907</x:v>
+        <x:f>INDEX('Previous 30 Crosscheck'!$E$8:$E$37,MATCH($B13,'Previous 30 Crosscheck'!$A$8:$A$37,0))</x:f>
+        <x:v>101.23457410318274</x:v>
       </x:c>
       <x:c r="E13" s="19" t="str">
-        <x:f>INDEX('Additional Leads'!$I$8:$I$30,MATCH($B13,'Additional Leads'!$A$8:$A$30,0))</x:f>
-        <x:v>434-208-8602</x:v>
+        <x:f>INDEX('Previous 30 Crosscheck'!$J$8:$J$37,MATCH($B13,'Previous 30 Crosscheck'!$A$8:$A$37,0))</x:f>
+        <x:v>704-933-7550</x:v>
       </x:c>
       <x:c r="F13" s="11" t="str">
-        <x:v>New individual lead; own site offers pork processing and animal sourcing.</x:v>
+        <x:v>Inspected market-hog prospect inside the radius. Documented fit merits priority despite limited web presence.</x:v>
       </x:c>
       <x:c r="G13" s="11" t="str">
         <x:v>Both unknown</x:v>
       </x:c>
       <x:c r="H13" s="11" t="str">
-        <x:v>https://easternviewfarmsllc.com/</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="45" customHeight="1">
+        <x:v>No company website confirmed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="58" customHeight="1">
       <x:c r="A14" s="17" t="n">
         <x:v>7</x:v>
       </x:c>
       <x:c r="B14" s="12" t="str">
-        <x:v>Gale McLamb Meats</x:v>
+        <x:v>Key Packing Company</x:v>
       </x:c>
       <x:c r="C14" s="16" t="n">
         <x:f>INDEX('Previous 30 Crosscheck'!$D$8:$D$37,MATCH($B14,'Previous 30 Crosscheck'!$A$8:$A$37,0))</x:f>
-        <x:v>59.73757009067048</x:v>
+        <x:v>69.72269446432833</x:v>
       </x:c>
       <x:c r="D14" s="16" t="n">
         <x:f>INDEX('Previous 30 Crosscheck'!$E$8:$E$37,MATCH($B14,'Previous 30 Crosscheck'!$A$8:$A$37,0))</x:f>
-        <x:v>48.036921080446234</x:v>
+        <x:v>52.88887432349344</x:v>
       </x:c>
       <x:c r="E14" s="17" t="str">
         <x:f>INDEX('Previous 30 Crosscheck'!$J$8:$J$37,MATCH($B14,'Previous 30 Crosscheck'!$A$8:$A$37,0))</x:f>
-        <x:v>910-892-7279</x:v>
+        <x:v>910-464-3507</x:v>
       </x:c>
       <x:c r="F14" s="12" t="str">
-        <x:v>Nearby state-inspected cattle and swine slaughter.</x:v>
+        <x:v>State-inspected swine slaughter within practical driving distance. Space and suitable volume unconfirmed.</x:v>
       </x:c>
       <x:c r="G14" s="12" t="str">
         <x:v>Both unknown</x:v>
@@ -782,27 +807,27 @@
         <x:v>No company website confirmed</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="45" customHeight="1">
+    <x:row r="15" ht="58" customHeight="1">
       <x:c r="A15" s="19" t="n">
         <x:v>8</x:v>
       </x:c>
       <x:c r="B15" s="11" t="str">
-        <x:v>Key Packing Company</x:v>
+        <x:v>Quaqua Creek Farm</x:v>
       </x:c>
       <x:c r="C15" s="18" t="n">
         <x:f>INDEX('Previous 30 Crosscheck'!$D$8:$D$37,MATCH($B15,'Previous 30 Crosscheck'!$A$8:$A$37,0))</x:f>
-        <x:v>69.72269446432833</x:v>
+        <x:v>67.20309641692515</x:v>
       </x:c>
       <x:c r="D15" s="18" t="n">
         <x:f>INDEX('Previous 30 Crosscheck'!$E$8:$E$37,MATCH($B15,'Previous 30 Crosscheck'!$A$8:$A$37,0))</x:f>
-        <x:v>52.88887432349344</x:v>
+        <x:v>48.35204925832898</x:v>
       </x:c>
       <x:c r="E15" s="19" t="str">
         <x:f>INDEX('Previous 30 Crosscheck'!$J$8:$J$37,MATCH($B15,'Previous 30 Crosscheck'!$A$8:$A$37,0))</x:f>
-        <x:v>910-464-3507</x:v>
+        <x:v>336-939-2656</x:v>
       </x:c>
       <x:c r="F15" s="11" t="str">
-        <x:v>State-inspected multi-species plant within practical driving distance.</x:v>
+        <x:v>State-inspected swine listing and short drive. Missing volume data does not earn a higher score.</x:v>
       </x:c>
       <x:c r="G15" s="11" t="str">
         <x:v>Both unknown</x:v>
@@ -811,68 +836,122 @@
         <x:v>No company website confirmed</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="45" customHeight="1">
+    <x:row r="16" ht="58" customHeight="1">
       <x:c r="A16" s="17" t="n">
         <x:v>9</x:v>
       </x:c>
       <x:c r="B16" s="12" t="str">
-        <x:v>Quaqua Creek Farm</x:v>
+        <x:v>Farmington Meat Processing</x:v>
       </x:c>
       <x:c r="C16" s="16" t="n">
-        <x:f>INDEX('Previous 30 Crosscheck'!$D$8:$D$37,MATCH($B16,'Previous 30 Crosscheck'!$A$8:$A$37,0))</x:f>
-        <x:v>67.20309641692515</x:v>
+        <x:f>INDEX('Additional Leads'!$C$8:$C$30,MATCH($B16,'Additional Leads'!$A$8:$A$30,0))</x:f>
+        <x:v>102.58086524695776</x:v>
       </x:c>
       <x:c r="D16" s="16" t="n">
-        <x:f>INDEX('Previous 30 Crosscheck'!$E$8:$E$37,MATCH($B16,'Previous 30 Crosscheck'!$A$8:$A$37,0))</x:f>
-        <x:v>48.35204925832898</x:v>
+        <x:f>INDEX('Additional Leads'!$D$8:$D$30,MATCH($B16,'Additional Leads'!$A$8:$A$30,0))</x:f>
+        <x:v>91.65576089158736</x:v>
       </x:c>
       <x:c r="E16" s="17" t="str">
-        <x:f>INDEX('Previous 30 Crosscheck'!$J$8:$J$37,MATCH($B16,'Previous 30 Crosscheck'!$A$8:$A$37,0))</x:f>
-        <x:v>336-939-2656</x:v>
+        <x:f>INDEX('Additional Leads'!$I$8:$I$30,MATCH($B16,'Additional Leads'!$A$8:$A$30,0))</x:f>
+        <x:v>336-998-7092</x:v>
       </x:c>
       <x:c r="F16" s="12" t="str">
-        <x:v>State-inspected swine listing; closer than many western candidates.</x:v>
+        <x:v>State directory and social descriptions corroborate pig processing. Volume remains unknown.</x:v>
       </x:c>
       <x:c r="G16" s="12" t="str">
         <x:v>Both unknown</x:v>
       </x:c>
       <x:c r="H16" s="12" t="str">
-        <x:v>No company website confirmed</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="45" customHeight="1">
+        <x:v>https://www.facebook.com/FarmingtonMeat/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="58" customHeight="1">
       <x:c r="A17" s="19" t="n">
         <x:v>10</x:v>
       </x:c>
       <x:c r="B17" s="11" t="str">
-        <x:v>Cool Springs Farm and Meat</x:v>
+        <x:v>Contentnea Farms</x:v>
       </x:c>
       <x:c r="C17" s="18" t="n">
         <x:f>INDEX('Previous 30 Crosscheck'!$D$8:$D$37,MATCH($B17,'Previous 30 Crosscheck'!$A$8:$A$37,0))</x:f>
-        <x:v>106.77114401892945</x:v>
+        <x:v>90.29008092738407</x:v>
       </x:c>
       <x:c r="D17" s="18" t="n">
         <x:f>INDEX('Previous 30 Crosscheck'!$E$8:$E$37,MATCH($B17,'Previous 30 Crosscheck'!$A$8:$A$37,0))</x:f>
-        <x:v>98.31805633055046</x:v>
+        <x:v>72.64760579541328</x:v>
       </x:c>
       <x:c r="E17" s="19" t="str">
         <x:f>INDEX('Previous 30 Crosscheck'!$J$8:$J$37,MATCH($B17,'Previous 30 Crosscheck'!$A$8:$A$37,0))</x:f>
-        <x:v>336-835-5377</x:v>
+        <x:v>252-289-3083</x:v>
       </x:c>
       <x:c r="F17" s="11" t="str">
-        <x:v>Inspected hog slaughter with a public booking page.</x:v>
+        <x:v>Inspected pork processing is documented. Follow stronger-fit calls while qualifying suitable pig availability.</x:v>
       </x:c>
       <x:c r="G17" s="11" t="str">
         <x:v>Both unknown</x:v>
       </x:c>
       <x:c r="H17" s="11" t="str">
-        <x:v>https://www.csmpfarmstore.com/</x:v>
-      </x:c>
+        <x:v>https://contentneafarms.com/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="29" customHeight="1">
+      <x:c r="A19" s="22" t="str">
+        <x:v>EcoFriendly #4 is an early supplier-performed harvesting discussion. Its aggregate slaughter category does not establish weekly pig volume.</x:v>
+      </x:c>
+      <x:c r="B19" s="22"/>
+      <x:c r="C19" s="22"/>
+      <x:c r="D19" s="22"/>
+      <x:c r="E19" s="22"/>
+      <x:c r="F19" s="22"/>
+      <x:c r="G19" s="22"/>
+      <x:c r="H19" s="22"/>
+    </x:row>
+    <x:row r="20" ht="29" customHeight="1">
+      <x:c r="A20" s="22" t="str">
+        <x:v>Conditional complementary choices: EcoFriendly, Select and Farmington, if Purchasing selects Piedmont, McLamb’s Benson and Gale McLamb.</x:v>
+      </x:c>
+      <x:c r="B20" s="22"/>
+      <x:c r="C20" s="22"/>
+      <x:c r="D20" s="22"/>
+      <x:c r="E20" s="22"/>
+      <x:c r="F20" s="22"/>
+      <x:c r="G20" s="22"/>
+      <x:c r="H20" s="22"/>
+    </x:row>
+    <x:row r="21" ht="29" customHeight="1">
+      <x:c r="A21" s="22" t="str">
+        <x:v>First call question: How many pigs in the 140–220-pound live-weight range do you actually slaughter in a typical week?</x:v>
+      </x:c>
+      <x:c r="B21" s="22"/>
+      <x:c r="C21" s="22"/>
+      <x:c r="D21" s="22"/>
+      <x:c r="E21" s="22"/>
+      <x:c r="F21" s="22"/>
+      <x:c r="G21" s="22"/>
+      <x:c r="H21" s="22"/>
+    </x:row>
+    <x:row r="22" ht="29" customHeight="1">
+      <x:c r="A22" s="22" t="str">
+        <x:v>Then confirm operation, tissue ownership, harvesting staff or crew space, collection timing, chilling and commercial terms.</x:v>
+      </x:c>
+      <x:c r="B22" s="22"/>
+      <x:c r="C22" s="22"/>
+      <x:c r="D22" s="22"/>
+      <x:c r="E22" s="22"/>
+      <x:c r="F22" s="22"/>
+      <x:c r="G22" s="22"/>
+      <x:c r="H22" s="22"/>
     </x:row>
   </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A19:H19"/>
+    <x:mergeCell ref="A20:H20"/>
+    <x:mergeCell ref="A21:H21"/>
+    <x:mergeCell ref="A22:H22"/>
+  </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R91df91b764c74fe7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R722fb03f13b84118"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -903,7 +982,7 @@
     </x:row>
     <x:row r="2" ht="22" customHeight="1">
       <x:c r="A2" s="4" t="str">
-        <x:v>Fact review against Claude’s current study</x:v>
+        <x:v>Fact review and recommendation changes</x:v>
       </x:c>
       <x:c r="B2" s="5"/>
       <x:c r="C2" s="5"/>
@@ -927,7 +1006,7 @@
     </x:row>
     <x:row r="4" ht="22" customHeight="1">
       <x:c r="A4" s="6" t="str">
-        <x:v>Checked September 28, 2026, including Claude’s concurrent update. Unknown means unconfirmed, not zero.</x:v>
+        <x:v>Baseline comparison retained. Revision 2.1 adds ranking changes and later Rocksteady updates.</x:v>
       </x:c>
       <x:c r="B4" s="2"/>
       <x:c r="C4" s="2"/>
@@ -1023,13 +1102,13 @@
         <x:v>120 miles used as a road-distance gate.</x:v>
       </x:c>
       <x:c r="E9" s="11" t="str">
-        <x:v>Literal 120-mile radius and a 120-mile drive are different. Both are now shown.</x:v>
+        <x:v>The user specified a 120-mile radius. Road mileage measures logistics and must not independently exclude an in-radius supplier.</x:v>
       </x:c>
       <x:c r="F9" s="11" t="str">
-        <x:v>EcoFriendly: 92.6 radial / 120.4 road. Acre: 119.7 / 141.1; boundary depends on actual base.</x:v>
+        <x:v>EcoFriendly qualifies geographically at 92.6 radial miles. Its 120.4-mile drive informs collection cost and inspection planning.</x:v>
       </x:c>
       <x:c r="G9" s="11" t="str">
-        <x:v>Clarified definition</x:v>
+        <x:v>Ranking rule corrected</x:v>
       </x:c>
       <x:c r="H9" s="11" t="str">
         <x:v>https://project-osrm.org/</x:v>
@@ -1057,9 +1136,7 @@
       <x:c r="G10" s="12" t="str">
         <x:v>Resolved by concurrent Claude update</x:v>
       </x:c>
-      <x:c r="H10" s="12" t="str">
-        <x:v>User-stated requirements / research scope</x:v>
-      </x:c>
+      <x:c r="H10" s="12" t="str"/>
     </x:row>
     <x:row r="11" ht="55.5" customHeight="1">
       <x:c r="A11" s="11" t="str">
@@ -1083,9 +1160,7 @@
       <x:c r="G11" s="11" t="str">
         <x:v>Preference aligned; absence not proven</x:v>
       </x:c>
-      <x:c r="H11" s="11" t="str">
-        <x:v>User-stated requirements / research scope</x:v>
-      </x:c>
+      <x:c r="H11" s="11" t="str"/>
     </x:row>
     <x:row r="12" ht="55.5" customHeight="1">
       <x:c r="A12" s="12" t="str">
@@ -1121,19 +1196,19 @@
         <x:v>Weekly arithmetic</x:v>
       </x:c>
       <x:c r="C13" s="11" t="str">
-        <x:v>Sources &amp; Confidence row 7</x:v>
+        <x:v>Sources &amp; Confidence row 7 (baseline comparison)</x:v>
       </x:c>
       <x:c r="D13" s="11" t="str">
         <x:v>Category 3 upper ceiling ~1,917/week.</x:v>
       </x:c>
       <x:c r="E13" s="11" t="str">
-        <x:v>A 360-day interval contains 360/7 weeks. 100,000 * 7/360 = 1,944.4 total heads/week at the exclusive boundary. Category 1 boundary 19.4; category 2 194.4.</x:v>
+        <x:v>A 360-day interval contains 360/7 weeks. 100,000 * 7/360 = 1,944.4 total heads/week at the exclusive boundary. Category 1 boundary 19.4; category 2 194.4. Subsequent Claude commit a403954 incorporated a related correction; this row preserves the original comparison.</x:v>
       </x:c>
       <x:c r="F13" s="11" t="str">
         <x:v>Even corrected average bounds cannot cap current capacity or quantify pigs at a multi-species plant.</x:v>
       </x:c>
       <x:c r="G13" s="11" t="str">
-        <x:v>Corrected calculation</x:v>
+        <x:v>Addressed in later Claude update</x:v>
       </x:c>
       <x:c r="H13" s="11" t="str">
         <x:v>https://www.federalregister.gov/documents/2026/03/24/2026-05746/revising-establishment-size-definitions</x:v>
@@ -1251,19 +1326,19 @@
         <x:v>Farmington visibility</x:v>
       </x:c>
       <x:c r="C18" s="12" t="str">
-        <x:v>Supplier Roster row 74; absent from Beebop 30</x:v>
+        <x:v>Supplier Roster row 74; absent from Beebop 30 (baseline comparison)</x:v>
       </x:c>
       <x:c r="D18" s="12" t="str">
         <x:v>Only buried in state-plant group.</x:v>
       </x:c>
       <x:c r="E18" s="12" t="str">
-        <x:v>State P-381 includes swine slaughter; Facebook and Instagram describe pig processing. 102.6 road miles from Durham.</x:v>
+        <x:v>State P-381 includes swine slaughter; Facebook and Instagram describe pig processing. 102.6 road miles from Durham. Subsequent Claude commit a403954 incorporated a related correction; this row preserves the original comparison.</x:v>
       </x:c>
       <x:c r="F18" s="12" t="str">
         <x:v>Elevated to an individually documented qualification prospect. Not a newly discovered company relative to Claude.</x:v>
       </x:c>
       <x:c r="G18" s="12" t="str">
-        <x:v>Expanded known lead</x:v>
+        <x:v>Addressed in later Claude update</x:v>
       </x:c>
       <x:c r="H18" s="12" t="str">
         <x:v>https://www.ncagr.gov/divisions/meat-poultry-inspection/wplants/download?attachment=
@@ -1279,19 +1354,19 @@
         <x:v>Easternview and Butcher’s Block</x:v>
       </x:c>
       <x:c r="C19" s="11" t="str">
-        <x:v>Not named in reviewed Claude roster</x:v>
+        <x:v>Not named in reviewed Claude roster (baseline comparison)</x:v>
       </x:c>
       <x:c r="D19" s="11" t="str">
         <x:v>No individual records.</x:v>
       </x:c>
       <x:c r="E19" s="11" t="str">
-        <x:v>Two additional Virginia candidates within 76 road miles. Easternview has direct company corroboration; Butcher’s Block has directory mirror plus Virginia processor listing.</x:v>
+        <x:v>Two additional Virginia candidates within 76 road miles. Easternview has direct company corroboration; Butcher’s Block has directory mirror plus Virginia processor listing. Subsequent Claude commit a403954 incorporated a related correction; this row preserves the original comparison.</x:v>
       </x:c>
       <x:c r="F19" s="11" t="str">
         <x:v>Potential small-scale supplements. Current pig volume and research operations remain unverified.</x:v>
       </x:c>
       <x:c r="G19" s="11" t="str">
-        <x:v>New documented leads</x:v>
+        <x:v>Addressed in later Claude update</x:v>
       </x:c>
       <x:c r="H19" s="11" t="str">
         <x:v>https://easternviewfarmsllc.com/
@@ -1334,19 +1409,19 @@
         <x:v>Godwin closure claim</x:v>
       </x:c>
       <x:c r="C21" s="11" t="str">
-        <x:v>Supplier Roster row 122</x:v>
+        <x:v>Supplier Roster row 122 (baseline comparison)</x:v>
       </x:c>
       <x:c r="D21" s="11" t="str">
         <x:v>Inactive Altoona, Iowa M760A used alongside directory absence to declare Godwin closed.</x:v>
       </x:c>
       <x:c r="E21" s="11" t="str">
-        <x:v>Claude’s latest workbook retains the Godwin closure conclusion. Iowa M760A cannot establish North Carolina site closure. Carrier and association listings cannot prove current slaughter either.</x:v>
+        <x:v>Claude’s latest workbook retains the Godwin closure conclusion. Iowa M760A cannot establish North Carolina site closure. Carrier and association listings cannot prove current slaughter either. Subsequent Claude commit a403954 incorporated a related correction; this row preserves the original comparison.</x:v>
       </x:c>
       <x:c r="F21" s="11" t="str">
         <x:v>Godwin remains unresolved and outside the priority shortlist; no reopening or closure conclusion in this pass.</x:v>
       </x:c>
       <x:c r="G21" s="11" t="str">
-        <x:v>Unsupported cross-site inference</x:v>
+        <x:v>Addressed in later Claude update</x:v>
       </x:c>
       <x:c r="H21" s="11" t="str">
         <x:v>https://www.ncmpa.com/associate-members/
@@ -1361,19 +1436,19 @@
         <x:v>Mitchell facility identity</x:v>
       </x:c>
       <x:c r="C22" s="12" t="str">
-        <x:v>Supplier Roster rows 14 and 86</x:v>
+        <x:v>Supplier Roster rows 14 and 86 (baseline comparison)</x:v>
       </x:c>
       <x:c r="D22" s="12" t="str">
         <x:v>King M46822B inactive and Walnut Cove historical concern.</x:v>
       </x:c>
       <x:c r="E22" s="12" t="str">
-        <x:v>September state directory lists Walnut Cove TA-46822. King and Walnut Cove are separate establishment identities. Historical handling allegation not independently revalidated.</x:v>
+        <x:v>September state directory lists Walnut Cove TA-46822. King and Walnut Cove are separate establishment identities. Historical handling allegation not independently revalidated. Subsequent Claude commit a403954 incorporated a related correction; this row preserves the original comparison.</x:v>
       </x:c>
       <x:c r="F22" s="12" t="str">
         <x:v>Separate current plant status from other-site closure and from unresolved historical quality evidence.</x:v>
       </x:c>
       <x:c r="G22" s="12" t="str">
-        <x:v>Identity clarified; concern unresolved</x:v>
+        <x:v>Addressed in later Claude update</x:v>
       </x:c>
       <x:c r="H22" s="12" t="str">
         <x:v>https://www.ncagr.gov/divisions/meat-poultry-inspection/wplants/download?attachment=
@@ -1388,19 +1463,19 @@
         <x:v>Bass internal inconsistency</x:v>
       </x:c>
       <x:c r="C23" s="11" t="str">
-        <x:v>Supplier Roster row 23 D/F; Rated Candidates row 12</x:v>
+        <x:v>Supplier Roster row 23 D/F; Rated Candidates row 12 (baseline comparison)</x:v>
       </x:c>
       <x:c r="D23" s="11" t="str">
         <x:v>Both category 1 and category 2 appear; grant date treated as new kill floor.</x:v>
       </x:c>
       <x:c r="E23" s="11" t="str">
-        <x:v>Current state directory confirms slaughter only. Category change not independently verified. Grant dates may reflect administrative changes.</x:v>
+        <x:v>Current state directory confirms slaughter only. Category change not independently verified. Grant dates may reflect administrative changes. Subsequent Claude commit a403954 incorporated a related correction; this row preserves the original comparison.</x:v>
       </x:c>
       <x:c r="F23" s="11" t="str">
         <x:v>No verified growth rate, new floor date or current weekly count.</x:v>
       </x:c>
       <x:c r="G23" s="11" t="str">
-        <x:v>Workbook conflict unresolved</x:v>
+        <x:v>Addressed in later Claude update</x:v>
       </x:c>
       <x:c r="H23" s="11" t="str">
         <x:v>https://www.ncagr.gov/divisions/meat-poultry-inspection/wplants/download?attachment=</x:v>
@@ -1534,9 +1609,7 @@
       <x:c r="G28" s="12" t="str">
         <x:v>Unconfirmed across new leads</x:v>
       </x:c>
-      <x:c r="H28" s="12" t="str">
-        <x:v>User-stated requirements / research scope</x:v>
-      </x:c>
+      <x:c r="H28" s="12" t="str"/>
     </x:row>
     <x:row r="29" ht="55.5" customHeight="1">
       <x:c r="A29" s="11" t="str">
@@ -1560,9 +1633,7 @@
       <x:c r="G29" s="11" t="str">
         <x:v>Outside verification scope</x:v>
       </x:c>
-      <x:c r="H29" s="11" t="str">
-        <x:v>User-stated requirements / research scope</x:v>
-      </x:c>
+      <x:c r="H29" s="11" t="str"/>
     </x:row>
     <x:row r="30" ht="55.5" customHeight="1">
       <x:c r="A30" s="12" t="str">
@@ -1572,28 +1643,107 @@
         <x:v>EcoFriendly exact facility distance</x:v>
       </x:c>
       <x:c r="C30" s="12" t="str">
-        <x:v>Supplier Roster row 41; Rated Candidates</x:v>
+        <x:v>Supplier Roster row 41; Rated Candidates (baseline comparison)</x:v>
       </x:c>
       <x:c r="D30" s="12" t="str">
         <x:v>Updated Claude: approximately 112 road miles, city-level geocode.</x:v>
       </x:c>
       <x:c r="E30" s="12" t="str">
-        <x:v>Exact address 3397 Stony Fork Road routes to 120.4 road miles and 92.6 radial miles from Durham City Hall.</x:v>
+        <x:v>Exact address 3397 Stony Fork Road routes to 120.4 road miles and 92.6 radial miles from Durham City Hall. Subsequent Claude commit a403954 incorporated a related correction; this row preserves the original comparison.</x:v>
       </x:c>
       <x:c r="F30" s="12" t="str">
         <x:v>Inside literal radius; just beyond a strict 120-road-mile screen. City-level distance is not sufficient near a boundary.</x:v>
       </x:c>
       <x:c r="G30" s="12" t="str">
-        <x:v>Facility-specific distance refinement</x:v>
+        <x:v>Addressed in later Claude update</x:v>
       </x:c>
       <x:c r="H30" s="12" t="str">
         <x:v>https://www.ecofriendly.com/services</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="140" customHeight="1">
+      <x:c r="A31" s="25" t="str">
+        <x:v>F24</x:v>
+      </x:c>
+      <x:c r="B31" s="25" t="str">
+        <x:v>Call ranking and missing-data bias</x:v>
+      </x:c>
+      <x:c r="C31" s="25" t="str">
+        <x:v>Beebop first ten; Rocksteady feedback supplied by user</x:v>
+      </x:c>
+      <x:c r="D31" s="25" t="str">
+        <x:v>EcoFriendly and Select were under-prioritized; small or unknown-volume plants received too much weight.</x:v>
+      </x:c>
+      <x:c r="E31" s="25" t="str">
+        <x:v>Accepted. EcoFriendly enters at #4 and Select at #6. Easternview and Cool Springs move to follow-up. Gale rises to #3. Missing information gives no positive ranking credit.</x:v>
+      </x:c>
+      <x:c r="F31" s="25" t="str">
+        <x:v>Priorities reflect documented fit and practical access. They do not imply confirmed scale or an accepted commercial agreement.</x:v>
+      </x:c>
+      <x:c r="G31" s="25" t="str">
+        <x:v>Recommendation revised</x:v>
+      </x:c>
+      <x:c r="H31" s="25" t="str">
+        <x:v>User-provided Rocksteady comparison, September 28, 2026
+https://www.ecofriendly.com/services</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="140" customHeight="1">
+      <x:c r="A32" s="25" t="str">
+        <x:v>F25</x:v>
+      </x:c>
+      <x:c r="B32" s="25" t="str">
+        <x:v>New statewide historical hog evidence</x:v>
+      </x:c>
+      <x:c r="C32" s="25" t="str">
+        <x:v>Claude commit 1cb841f; volume inference update</x:v>
+      </x:c>
+      <x:c r="D32" s="25" t="str">
+        <x:v>Virginia: 7,841 hogs across 16 federal plants in 2025. South Carolina: 14,070 across 8. Applied as hard caps.</x:v>
+      </x:c>
+      <x:c r="E32" s="25" t="str">
+        <x:v>The official 2025 table confirms those annual counts, in head. They are historical state aggregates. They are not current weekly plant volume, suitable-weight supply or capacity.</x:v>
+      </x:c>
+      <x:c r="F32" s="25" t="str">
+        <x:v>Weakens EcoFriendly’s volume-replacement case. Keep #4 as a supplier-performed harvesting discussion. No statewide total is entered as a plant count.</x:v>
+      </x:c>
+      <x:c r="G32" s="25" t="str">
+        <x:v>Source confirmed; inference limited</x:v>
+      </x:c>
+      <x:c r="H32" s="25" t="str">
+        <x:v>https://esmis.nal.usda.gov/sites/default/release-files/795870/lsan0426.txt</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="140" customHeight="1">
+      <x:c r="A33" s="25" t="str">
+        <x:v>F26</x:v>
+      </x:c>
+      <x:c r="B33" s="25" t="str">
+        <x:v>Qualification questions and selection split</x:v>
+      </x:c>
+      <x:c r="C33" s="25" t="str">
+        <x:v>Revised recommendation for Rocksteady</x:v>
+      </x:c>
+      <x:c r="D33" s="25" t="str">
+        <x:v>Suggested complementary selections: EcoFriendly, Select and Farmington.</x:v>
+      </x:c>
+      <x:c r="E33" s="25" t="str">
+        <x:v>Conditional on Purchasing selecting Piedmont, McLamb’s Benson and Gale. No assignments or contact results are recorded.</x:v>
+      </x:c>
+      <x:c r="F33" s="25" t="str">
+        <x:v>Ask current weekly pigs, 140–220-pound live-weight availability, organ ownership, trained harvesting or crew space, timing and chilling.</x:v>
+      </x:c>
+      <x:c r="G33" s="25" t="str">
+        <x:v>Conditional recommendation</x:v>
+      </x:c>
+      <x:c r="H33" s="25" t="str">
+        <x:v>User requirements and September 28 recommendation review</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R334582331c5d480e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf3cfbb35c1604ad7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1648,7 +1798,7 @@
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
       <x:c r="A3" s="6" t="str">
-        <x:v>Claude workbook references preserve the original claims. New review findings sit beside them.</x:v>
+        <x:v>Original ranks and Claude claims are historical. Current first-ten priorities appear in Review status.</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -1664,7 +1814,7 @@
     </x:row>
     <x:row r="4" ht="22" customHeight="1">
       <x:c r="A4" s="6" t="str">
-        <x:v>Checked September 28, 2026, including Claude’s concurrent update. Unknown means unconfirmed, not zero.</x:v>
+        <x:v>Revision 2.1, September 28, 2026. Original comparison snapshot: 5c3d169. Later corrections are in Fact Review.</x:v>
       </x:c>
       <x:c r="B4" s="2"/>
       <x:c r="C4" s="2"/>
@@ -1711,7 +1861,7 @@
         <x:v>Supplier</x:v>
       </x:c>
       <x:c r="B7" s="10" t="str">
-        <x:v>Prior rank</x:v>
+        <x:v>Original rank</x:v>
       </x:c>
       <x:c r="C7" s="10" t="str">
         <x:v>Claude location</x:v>
@@ -1769,10 +1919,10 @@
 (FSIS cat 2 ceiling)</x:v>
       </x:c>
       <x:c r="H8" s="12" t="str">
-        <x:v>Retain qualification lead</x:v>
+        <x:v>First 10: #1</x:v>
       </x:c>
       <x:c r="I8" s="12" t="str">
-        <x:v>Claude’s new Durham value (~48 road miles) agrees with Beebop’s 47.8. Published 150 lb live minimum only partly overlaps target. Disposal fee does not establish ownership or availability of particular organs.</x:v>
+        <x:v>Claude’s new Durham value (~48 road miles) agrees with Beebop’s 47.8. Published 150 lb live minimum only partly overlaps target. Disposal fee does not establish ownership or availability of particular organs. Revised priority: Published 150-pound live minimum overlaps the target; custom processing and nearby slaughter site.</x:v>
       </x:c>
       <x:c r="J8" s="12" t="str">
         <x:v>336-628-4949</x:v>
@@ -1809,10 +1959,10 @@
 publish no volumes</x:v>
       </x:c>
       <x:c r="H9" s="11" t="str">
-        <x:v>Retain qualification lead</x:v>
+        <x:v>First 10: #2</x:v>
       </x:c>
       <x:c r="I9" s="11" t="str">
-        <x:v>State P-247 identity, address and phone match Lee’s Fresh Market. Durham distance now agrees. Company website and social signals support processing activity; pig volume and room remain unknown.</x:v>
+        <x:v>State P-247 identity, address and phone match Lee’s Fresh Market. Durham distance now agrees. Company website and social signals support processing activity; pig volume and room remain unknown. Revised priority: Nearby inspected swine plant with matching company identity. Practical early qualification prospect.</x:v>
       </x:c>
       <x:c r="J9" s="11" t="str">
         <x:v>919-894-2587</x:v>
@@ -1849,10 +1999,10 @@
 (FSIS cat 2 ceiling)</x:v>
       </x:c>
       <x:c r="H10" s="12" t="str">
-        <x:v>Retain qualification lead</x:v>
+        <x:v>First 10: #5</x:v>
       </x:c>
       <x:c r="I10" s="12" t="str">
-        <x:v>One Flowers establishment, M21747. Claude correctly labels its George Flowers row as duplicate. Count once. No actual weekly volume published.</x:v>
+        <x:v>One Flowers establishment, M21747. Claude correctly labels its George Flowers row as duplicate. Count once. No actual weekly volume published. Revised priority: Nearby documented hog slaughter. George Flowers is the same plant and is counted once.</x:v>
       </x:c>
       <x:c r="J10" s="12" t="str">
         <x:v>252-237-2982</x:v>
@@ -1889,10 +2039,10 @@
 (FSIS cat 1)</x:v>
       </x:c>
       <x:c r="H11" s="11" t="str">
-        <x:v>Retain qualification lead</x:v>
+        <x:v>First 10: #10</x:v>
       </x:c>
       <x:c r="I11" s="11" t="str">
-        <x:v>State directory corroborates TA-2583, swine and Walstonburg kill site. Company public phone differs from directory: retain 252-289-3083 and 252-717-9229. Claude category-1-derived weekly figure is historical aggregate, not current pig count.</x:v>
+        <x:v>State directory corroborates TA-2583, swine and Walstonburg kill site. Company public phone differs from directory: retain 252-289-3083 and 252-717-9229. Claude category-1-derived weekly figure is historical aggregate, not current pig count. Revised priority: Inspected pork processing is documented. Follow stronger-fit calls while qualifying suitable pig availability.</x:v>
       </x:c>
       <x:c r="J11" s="11" t="str">
         <x:v>252-289-3083</x:v>
@@ -1929,10 +2079,10 @@
 retail-butcher scale</x:v>
       </x:c>
       <x:c r="H12" s="12" t="str">
-        <x:v>Retain qualification lead</x:v>
+        <x:v>First 10: #3</x:v>
       </x:c>
       <x:c r="I12" s="12" t="str">
-        <x:v>State directory corroborates swine slaughter and identity. Claude’s updated Durham distance agrees. Exact weekly pigs, suitable weights and room remain unknown.</x:v>
+        <x:v>State directory corroborates swine slaughter and identity. Claude’s updated Durham distance agrees. Exact weekly pigs, suitable weights and room remain unknown. Revised priority: Nearby state-inspected swine slaughter; practical Benson/Dunn visit grouping. No volume advantage assumed.</x:v>
       </x:c>
       <x:c r="J12" s="12" t="str">
         <x:v>910-892-7279</x:v>
@@ -1966,10 +2116,10 @@
         <x:v>unknown (small)</x:v>
       </x:c>
       <x:c r="H13" s="11" t="str">
-        <x:v>Retain qualification lead</x:v>
+        <x:v>First 10: #7</x:v>
       </x:c>
       <x:c r="I13" s="11" t="str">
-        <x:v>State directory corroborates swine slaughter and identity. Claude’s updated Durham distance agrees. Exact weekly pigs, suitable weights and room remain unknown.</x:v>
+        <x:v>State directory corroborates swine slaughter and identity. Claude’s updated Durham distance agrees. Exact weekly pigs, suitable weights and room remain unknown. Revised priority: State-inspected swine slaughter within practical driving distance. Space and suitable volume unconfirmed.</x:v>
       </x:c>
       <x:c r="J13" s="11" t="str">
         <x:v>910-464-3507</x:v>
@@ -2003,10 +2153,10 @@
         <x:v>unknown — state plants publish no volumes</x:v>
       </x:c>
       <x:c r="H14" s="12" t="str">
-        <x:v>Retain qualification lead</x:v>
+        <x:v>First 10: #8</x:v>
       </x:c>
       <x:c r="I14" s="12" t="str">
-        <x:v>State directory corroborates swine slaughter and identity. Claude’s updated Durham distance agrees. Exact weekly pigs, suitable weights and room remain unknown.</x:v>
+        <x:v>State directory corroborates swine slaughter and identity. Claude’s updated Durham distance agrees. Exact weekly pigs, suitable weights and room remain unknown. Revised priority: State-inspected swine listing and short drive. Missing volume data does not earn a higher score.</x:v>
       </x:c>
       <x:c r="J14" s="12" t="str">
         <x:v>336-939-2656</x:v>
@@ -2040,10 +2190,10 @@
         <x:v>&lt;19/wk (FSIS cat 1)</x:v>
       </x:c>
       <x:c r="H15" s="11" t="str">
-        <x:v>Retain qualification lead</x:v>
+        <x:v>Follow-up: outside first 10</x:v>
       </x:c>
       <x:c r="I15" s="11" t="str">
-        <x:v>State directory corroborates swine slaughter and identity. Claude’s updated Durham distance agrees. Exact weekly pigs, suitable weights and room remain unknown.</x:v>
+        <x:v>State directory corroborates swine slaughter and identity. Claude’s updated Durham distance agrees. Exact weekly pigs, suitable weights and room remain unknown. Moved out of the first ten. Useful small-volume alternative; public booking capability does not establish target volume.</x:v>
       </x:c>
       <x:c r="J15" s="11" t="str">
         <x:v>336-835-5377</x:v>
@@ -2400,10 +2550,10 @@
 (FSIS cat 2)</x:v>
       </x:c>
       <x:c r="H24" s="12" t="str">
-        <x:v>Retain qualification lead</x:v>
+        <x:v>First 10: #6</x:v>
       </x:c>
       <x:c r="I24" s="12" t="str">
-        <x:v>State directory corroborates swine slaughter and identity. Claude’s updated Durham distance agrees. Exact weekly pigs, suitable weights and room remain unknown.</x:v>
+        <x:v>State directory corroborates swine slaughter and identity. Claude’s updated Durham distance agrees. Exact weekly pigs, suitable weights and room remain unknown. Revised priority: Inspected market-hog prospect inside the radius. Documented fit merits priority despite limited web presence.</x:v>
       </x:c>
       <x:c r="J24" s="12" t="str">
         <x:v>704-933-7550</x:v>
@@ -2923,7 +3073,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd20698fb910f4094"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f9216a812fd43a5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3018,7 +3168,7 @@
     </x:row>
     <x:row r="4" ht="22" customHeight="1">
       <x:c r="A4" s="6" t="str">
-        <x:v>Checked September 28, 2026, including Claude’s concurrent update. Unknown means unconfirmed, not zero.</x:v>
+        <x:v>Revision 2.1: radius determines eligibility. Driving distance informs effort, not a separate exclusion.</x:v>
       </x:c>
       <x:c r="B4" s="2"/>
       <x:c r="C4" s="2"/>
@@ -3099,7 +3249,7 @@
         <x:v>120-mile radius</x:v>
       </x:c>
       <x:c r="F7" s="10" t="str">
-        <x:v>120-mile drive</x:v>
+        <x:v>Driving distance only</x:v>
       </x:c>
       <x:c r="G7" s="10" t="str">
         <x:v>Inspection / identity</x:v>
@@ -3143,7 +3293,7 @@
         <x:v>Farmington Meat Processing</x:v>
       </x:c>
       <x:c r="B8" s="12" t="str">
-        <x:v>High: additional qualification call</x:v>
+        <x:v>First 10: #9</x:v>
       </x:c>
       <x:c r="C8" s="16" t="n">
         <x:v>102.58086524695776</x:v>
@@ -3172,7 +3322,7 @@
         <x:v>https://www.facebook.com/FarmingtonMeat/</x:v>
       </x:c>
       <x:c r="K8" s="12" t="str">
-        <x:v>Claude row 74 grouped mention; absent from prior Beebop 30</x:v>
+        <x:v>Initially a grouped mention; Claude added an individual record in a403954 after Beebop round 2.</x:v>
       </x:c>
       <x:c r="L8" s="12" t="str">
         <x:v>State-inspected swine slaughter plus Facebook and Instagram pig-processing descriptions.</x:v>
@@ -3201,7 +3351,7 @@
         <x:v>Easternview Farms</x:v>
       </x:c>
       <x:c r="B9" s="11" t="str">
-        <x:v>High: additional qualification call</x:v>
+        <x:v>Follow-up: small-volume supplement</x:v>
       </x:c>
       <x:c r="C9" s="18" t="n">
         <x:v>75.973440109759</x:v>
@@ -3230,7 +3380,7 @@
         <x:v>https://easternviewfarmsllc.com/</x:v>
       </x:c>
       <x:c r="K9" s="11" t="str">
-        <x:v>Not named in reviewed Claude roster or prior Beebop 30</x:v>
+        <x:v>New in Beebop round 2; Claude added an individual record in a403954.</x:v>
       </x:c>
       <x:c r="L9" s="11" t="str">
         <x:v>Own site advertises pork processing, sourced animals and M1908. Directly describes on-site slaughter handling.</x:v>
@@ -3259,7 +3409,7 @@
         <x:v>The Butcher’s Block</x:v>
       </x:c>
       <x:c r="B10" s="12" t="str">
-        <x:v>Medium: additional qualification call</x:v>
+        <x:v>Follow-up: small-volume supplement</x:v>
       </x:c>
       <x:c r="C10" s="16" t="n">
         <x:v>73.9988467350672</x:v>
@@ -3288,7 +3438,7 @@
         <x:v>https://www.facebook.com/p/The-Butchers-Block-100057234168268/</x:v>
       </x:c>
       <x:c r="K10" s="12" t="str">
-        <x:v>Not named in reviewed Claude roster or prior Beebop 30</x:v>
+        <x:v>Newly documented in round 2; Claude added an individual record in a403954.</x:v>
       </x:c>
       <x:c r="L10" s="12" t="str">
         <x:v>Directory mirror lists hog slaughter M763; Virginia processor list independently matches address, phone and Facebook page.</x:v>
@@ -3370,12 +3520,12 @@
         <x:v>https://router.project-osrm.org/route/v1/driving/-78.899684,35.996069;-80.734541,35.618054?overview=false</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="69" customHeight="1">
+    <x:row r="12" ht="145" customHeight="1">
       <x:c r="A12" s="12" t="str">
         <x:v>EcoFriendly Foods</x:v>
       </x:c>
       <x:c r="B12" s="12" t="str">
-        <x:v>Medium: radius qualifies; longer drive</x:v>
+        <x:v>First 10: #4; supplier-performed harvesting discussion</x:v>
       </x:c>
       <x:c r="C12" s="16" t="n">
         <x:v>120.44771037143083</x:v>
@@ -3395,7 +3545,7 @@
         <x:v>M21938</x:v>
       </x:c>
       <x:c r="H12" s="12" t="str">
-        <x:v>M21938 reported by September 1 federal mirror; company claims federal inspection.</x:v>
+        <x:v>Category 3 is historical aggregate slaughter, not pigs/week. National Agricultural Statistics Service reports 7,841 federally inspected hogs across 16 Virginia plants in 2025. This is not EcoFriendly’s count or current capacity.</x:v>
       </x:c>
       <x:c r="I12" s="12" t="str">
         <x:v>540-525-0352</x:v>
@@ -3404,19 +3554,19 @@
         <x:v>https://www.ecofriendly.com/services</x:v>
       </x:c>
       <x:c r="K12" s="12" t="str">
-        <x:v>Claude row 41; September 28 revision gives ~112 road miles using city-level point. This pass refines exact plant address.</x:v>
+        <x:v>Claude row 41. Exact 120.4 road / 92.6 radial miles incorporated in a403954; 1cb841f adds state-total volume caution.</x:v>
       </x:c>
       <x:c r="L12" s="12" t="str">
         <x:v>Own services page offers slaughter and pork processing; published 2025 sheet includes small whole-hog harvest.</x:v>
       </x:c>
       <x:c r="M12" s="12" t="str">
-        <x:v>92.6 radial miles but 120.4 road miles. Broad category 3 includes other species including poultry. Pig-only count unknown; price-sheet carcass weights are not live weights.</x:v>
+        <x:v>Inside the 120-mile radius. Road distance affects logistics only. Current suitable pigs/week, operation, tissue rights and harvesting arrangements all remain unconfirmed.</x:v>
       </x:c>
       <x:c r="N12" s="12" t="str">
         <x:v>https://www.ecofriendly.com/_files/ugd/052161_5117723c9f1044eb8b0cda50b73d524f.pdf</x:v>
       </x:c>
       <x:c r="O12" s="12" t="str">
-        <x:v>https://www.ecofriendly.com/_files/ugd/052161_5117723c9f1044eb8b0cda50b73d524f.pdf</x:v>
+        <x:v>https://esmis.nal.usda.gov/sites/default/release-files/795870/lsan0426.txt</x:v>
       </x:c>
       <x:c r="P12" s="12" t="str">
         <x:v>3397 Stony Fork Road, Moneta, VA 24121</x:v>
@@ -3520,7 +3670,7 @@
         <x:v>https://www.kcfarmsva.com/kc-farms-meats</x:v>
       </x:c>
       <x:c r="K14" s="12" t="str">
-        <x:v>Not individually named in reviewed Claude roster or prior Beebop 30</x:v>
+        <x:v>Newly documented in round 2; Claude added an individual record in a403954.</x:v>
       </x:c>
       <x:c r="L14" s="12" t="str">
         <x:v>Own website confirms inspected on-farm processing but emphasizes beef; federal mirror lists hogs.</x:v>
@@ -4453,7 +4603,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R704c37cfd343420b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re02a69b0ebf24f48"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4693,7 +4843,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58bec7a11d83442d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R471016d3ff044504"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>